<commit_message>
add data into excel
</commit_message>
<xml_diff>
--- a/TestData/Testcase.xlsx
+++ b/TestData/Testcase.xlsx
@@ -62,7 +62,7 @@
             <color indexed="81"/>
             <sz val="10"/>
           </rPr>
-          <t>_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x000A_</t>
+          <t>_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x000A_</t>
         </r>
         <r>
           <rPr>
@@ -81,7 +81,7 @@
             <color indexed="81"/>
             <sz val="10"/>
           </rPr>
-          <t xml:space="preserve"> Những TCs phải được thực thi trong bất kỳ tình huống nào_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x000A_</t>
+          <t xml:space="preserve"> Những TCs phải được thực thi trong bất kỳ tình huống nào_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x000A_</t>
         </r>
         <r>
           <rPr>
@@ -100,7 +100,7 @@
             <color indexed="81"/>
             <sz val="10"/>
           </rPr>
-          <t xml:space="preserve"> Những TCs có thể được thực thi nếu thời gian cho phép._x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x000A_</t>
+          <t xml:space="preserve"> Những TCs có thể được thực thi nếu thời gian cho phép._x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x000A_</t>
         </r>
         <r>
           <rPr>
@@ -142,7 +142,7 @@
             <color indexed="81"/>
             <sz val="9"/>
           </rPr>
-          <t>_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x000A_Number of test cases to validate the specific test requirement</t>
+          <t>_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x000A_Number of test cases to validate the specific test requirement</t>
         </r>
       </text>
     </comment>
@@ -1025,7 +1025,7 @@
   </si>
   <si>
     <t xml:space="preserve">Transfer Complete!_x000D_
-$100.00 has been transferred from account #13677 to account #13899._x000D_
+$100.00 has been transferred from account #13899 to account #14121._x000D_
 See Account Activity for more details.</t>
   </si>
   <si>

</xml_diff>